<commit_message>
added new feature add ambulance call in smart hospital
</commit_message>
<xml_diff>
--- a/Python-Automation-SmartHospital/data_files/AddAmbulanceData.xlsx
+++ b/Python-Automation-SmartHospital/data_files/AddAmbulanceData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dhars\Documents\SmartHospitalPython\Python-Automation-SmartHospital\data_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F927F04D-5499-4251-A19C-D270F9B7A08D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E5F27D5-73E1-4DF2-A568-581B35981234}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4320" yWindow="3360" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{950A8404-7DD9-4EE0-89F1-F100EC1AAC03}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{950A8404-7DD9-4EE0-89F1-F100EC1AAC03}"/>
   </bookViews>
   <sheets>
     <sheet name="Validdata" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="12">
   <si>
     <t>vehicleno</t>
   </si>
@@ -65,6 +65,12 @@
   </si>
   <si>
     <t>Owned</t>
+  </si>
+  <si>
+    <t>MS07 DH 2001</t>
+  </si>
+  <si>
+    <t>Jagadeep</t>
   </si>
 </sst>
 </file>
@@ -423,7 +429,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CA9BEB5-0D2D-40F2-AE83-15F78A1E4111}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.77734375" customWidth="1"/>
@@ -471,6 +477,26 @@
         <v>9</v>
       </c>
     </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3">
+        <v>2025</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3">
+        <v>987654321</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -479,7 +505,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B422D4D6-E112-4E42-946F-A6330E7936C7}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.44140625" customWidth="1"/>
@@ -520,6 +546,23 @@
         <v>9</v>
       </c>
     </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>2025</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>987654321</v>
+      </c>
+      <c r="E3" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>